<commit_message>
updated teenclub templates to capture all data points into NDP
</commit_message>
<xml_diff>
--- a/teensclub_report.xlsx
+++ b/teensclub_report.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PIH\teenClub DHIS2 Integrator\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PIH\dhis2_excel_integrator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1E12963-6F61-4982-9B98-3D903DF7095A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FB1E045-AB2A-41AA-B3F9-7A1E4BCEB062}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" xr2:uid="{58AEABA8-2B34-4459-BB0A-42EC3882B367}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="34">
   <si>
     <t>Date</t>
   </si>
@@ -132,6 +132,12 @@
   </si>
   <si>
     <t>Facility</t>
+  </si>
+  <si>
+    <t>Teen Club - CD4 Drawn</t>
+  </si>
+  <si>
+    <t>Teen Club - Urine LAM Drawn</t>
   </si>
 </sst>
 </file>
@@ -269,7 +275,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -280,15 +286,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -322,6 +319,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -658,73 +658,79 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{199AE125-C6FD-41F1-8847-0C45D2D2C72F}">
-  <dimension ref="A1:S15"/>
+  <dimension ref="A1:U15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.08984375" customWidth="1"/>
-    <col min="2" max="2" width="10.453125" style="12" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="8.7265625" style="15"/>
+    <col min="2" max="2" width="10.453125" style="9" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.7265625" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="112.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:21" ht="112.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="17" t="s">
+      <c r="B1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D1" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="19" t="s">
+      <c r="G1" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="19" t="s">
+      <c r="H1" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="I1" s="19" t="s">
+      <c r="I1" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="J1" s="19" t="s">
+      <c r="J1" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="K1" s="19" t="s">
+      <c r="K1" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="L1" s="19" t="s">
+      <c r="L1" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="M1" s="19" t="s">
+      <c r="M1" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="N1" s="19" t="s">
+      <c r="N1" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="O1" s="19" t="s">
+      <c r="O1" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="19" t="s">
+      <c r="P1" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="Q1" s="20" t="s">
+      <c r="Q1" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="R1" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="S1" s="17" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="11">
-        <v>45638</v>
+      <c r="B2" s="8">
+        <v>45272</v>
       </c>
       <c r="C2" s="2">
         <v>95</v>
@@ -768,18 +774,24 @@
       <c r="P2" s="2">
         <v>0</v>
       </c>
-      <c r="Q2" s="14">
+      <c r="Q2" s="2">
+        <v>0</v>
+      </c>
+      <c r="R2" s="2">
+        <v>0</v>
+      </c>
+      <c r="S2" s="11">
         <f>D2+E2</f>
         <v>70</v>
       </c>
-      <c r="S2" s="8"/>
+      <c r="U2" s="5"/>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="11">
-        <v>45628</v>
+      <c r="B3" s="8">
+        <v>45262</v>
       </c>
       <c r="C3" s="2">
         <v>45</v>
@@ -823,18 +835,24 @@
       <c r="P3" s="2">
         <v>0</v>
       </c>
-      <c r="Q3" s="14">
-        <f t="shared" ref="Q3:Q15" si="0">D3+E3</f>
+      <c r="Q3" s="2">
+        <v>0</v>
+      </c>
+      <c r="R3" s="2">
+        <v>0</v>
+      </c>
+      <c r="S3" s="11">
+        <f t="shared" ref="S3:S15" si="0">D3+E3</f>
         <v>40</v>
       </c>
-      <c r="S3" s="8"/>
+      <c r="U3" s="5"/>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="11">
-        <v>45631</v>
+      <c r="B4" s="8">
+        <v>45265</v>
       </c>
       <c r="C4" s="2">
         <v>50</v>
@@ -876,20 +894,26 @@
         <v>1</v>
       </c>
       <c r="P4" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="2">
+        <v>0</v>
+      </c>
+      <c r="R4" s="2">
         <v>5</v>
       </c>
-      <c r="Q4" s="14">
+      <c r="S4" s="11">
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
-      <c r="S4" s="8"/>
+      <c r="U4" s="5"/>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="11">
-        <v>45635</v>
+      <c r="B5" s="8">
+        <v>45269</v>
       </c>
       <c r="C5" s="2">
         <v>15</v>
@@ -933,20 +957,26 @@
       <c r="P5" s="2">
         <v>0</v>
       </c>
-      <c r="Q5" s="14">
+      <c r="Q5" s="2">
+        <v>0</v>
+      </c>
+      <c r="R5" s="2">
+        <v>0</v>
+      </c>
+      <c r="S5" s="11">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="S5" s="8"/>
+      <c r="U5" s="5"/>
     </row>
-    <row r="6" spans="1:19" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:21" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="11">
-        <v>45635</v>
-      </c>
-      <c r="C6" s="5">
+      <c r="B6" s="8">
+        <v>45269</v>
+      </c>
+      <c r="C6" s="2">
         <v>90</v>
       </c>
       <c r="D6" s="2">
@@ -958,50 +988,56 @@
       <c r="F6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="2">
         <v>82</v>
       </c>
-      <c r="H6" s="5">
-        <v>0</v>
-      </c>
-      <c r="I6" s="5">
+      <c r="H6" s="2">
+        <v>0</v>
+      </c>
+      <c r="I6" s="2">
         <v>82</v>
       </c>
-      <c r="J6" s="5">
-        <v>0</v>
-      </c>
-      <c r="K6" s="5">
-        <v>0</v>
-      </c>
-      <c r="L6" s="5">
+      <c r="J6" s="2">
+        <v>0</v>
+      </c>
+      <c r="K6" s="2">
+        <v>0</v>
+      </c>
+      <c r="L6" s="2">
         <v>24</v>
       </c>
-      <c r="M6" s="5">
+      <c r="M6" s="2">
         <v>22</v>
       </c>
-      <c r="N6" s="5">
+      <c r="N6" s="2">
         <v>76</v>
       </c>
-      <c r="O6" s="5">
+      <c r="O6" s="2">
         <v>2</v>
       </c>
-      <c r="P6" s="6">
+      <c r="P6" s="2">
+        <v>9</v>
+      </c>
+      <c r="Q6" s="2">
+        <v>0</v>
+      </c>
+      <c r="R6" s="2">
         <v>24</v>
       </c>
-      <c r="Q6" s="14">
+      <c r="S6" s="11">
         <f t="shared" si="0"/>
         <v>82</v>
       </c>
-      <c r="S6" s="9"/>
+      <c r="U6" s="6"/>
     </row>
-    <row r="7" spans="1:19" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:21" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="11">
-        <v>45643</v>
-      </c>
-      <c r="C7" s="5">
+      <c r="B7" s="8">
+        <v>45277</v>
+      </c>
+      <c r="C7" s="2">
         <v>60</v>
       </c>
       <c r="D7" s="2">
@@ -1013,50 +1049,56 @@
       <c r="F7" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="2">
         <v>45</v>
       </c>
-      <c r="H7" s="5">
-        <v>0</v>
-      </c>
-      <c r="I7" s="5">
+      <c r="H7" s="2">
+        <v>0</v>
+      </c>
+      <c r="I7" s="2">
         <v>45</v>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="2">
         <v>3</v>
       </c>
-      <c r="K7" s="5">
+      <c r="K7" s="2">
         <v>3</v>
       </c>
-      <c r="L7" s="5">
+      <c r="L7" s="2">
         <v>6</v>
       </c>
-      <c r="M7" s="5">
+      <c r="M7" s="2">
         <v>6</v>
       </c>
-      <c r="N7" s="5">
+      <c r="N7" s="2">
         <v>37</v>
       </c>
-      <c r="O7" s="5">
-        <v>0</v>
-      </c>
-      <c r="P7" s="6">
+      <c r="O7" s="2">
+        <v>0</v>
+      </c>
+      <c r="P7" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>0</v>
+      </c>
+      <c r="R7" s="2">
         <v>12</v>
       </c>
-      <c r="Q7" s="14">
+      <c r="S7" s="11">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
-      <c r="S7" s="9"/>
+      <c r="U7" s="6"/>
     </row>
-    <row r="8" spans="1:19" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:21" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="11">
-        <v>45643</v>
-      </c>
-      <c r="C8" s="5">
+      <c r="B8" s="8">
+        <v>45277</v>
+      </c>
+      <c r="C8" s="2">
         <v>30</v>
       </c>
       <c r="D8" s="2">
@@ -1068,50 +1110,56 @@
       <c r="F8" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="2">
         <v>27</v>
       </c>
-      <c r="H8" s="5">
-        <v>0</v>
-      </c>
-      <c r="I8" s="5">
+      <c r="H8" s="2">
+        <v>0</v>
+      </c>
+      <c r="I8" s="2">
         <v>27</v>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="2">
         <v>4</v>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="2">
         <v>2</v>
       </c>
-      <c r="L8" s="5">
+      <c r="L8" s="2">
         <v>4</v>
       </c>
-      <c r="M8" s="5">
+      <c r="M8" s="2">
         <v>4</v>
       </c>
-      <c r="N8" s="5">
+      <c r="N8" s="2">
         <v>14</v>
       </c>
-      <c r="O8" s="5">
-        <v>0</v>
-      </c>
-      <c r="P8" s="7">
+      <c r="O8" s="2">
+        <v>0</v>
+      </c>
+      <c r="P8" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="2">
+        <v>2</v>
+      </c>
+      <c r="R8" s="2">
         <v>7</v>
       </c>
-      <c r="Q8" s="14">
+      <c r="S8" s="11">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="S8" s="10"/>
+      <c r="U8" s="7"/>
     </row>
-    <row r="9" spans="1:19" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:21" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="11">
-        <v>45628</v>
-      </c>
-      <c r="C9" s="5">
+      <c r="B9" s="8">
+        <v>45262</v>
+      </c>
+      <c r="C9" s="2">
         <v>80</v>
       </c>
       <c r="D9" s="2">
@@ -1123,48 +1171,54 @@
       <c r="F9" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="2">
         <v>59</v>
       </c>
-      <c r="H9" s="5">
-        <v>0</v>
-      </c>
-      <c r="I9" s="5">
+      <c r="H9" s="2">
+        <v>0</v>
+      </c>
+      <c r="I9" s="2">
         <v>59</v>
       </c>
-      <c r="J9" s="5">
-        <v>0</v>
-      </c>
-      <c r="K9" s="5">
-        <v>0</v>
-      </c>
-      <c r="L9" s="5">
+      <c r="J9" s="2">
+        <v>0</v>
+      </c>
+      <c r="K9" s="2">
+        <v>0</v>
+      </c>
+      <c r="L9" s="2">
         <v>8</v>
       </c>
-      <c r="M9" s="5">
+      <c r="M9" s="2">
         <v>8</v>
       </c>
-      <c r="N9" s="5">
+      <c r="N9" s="2">
         <v>36</v>
       </c>
-      <c r="O9" s="5">
-        <v>0</v>
-      </c>
-      <c r="P9" s="6">
+      <c r="O9" s="2">
+        <v>0</v>
+      </c>
+      <c r="P9" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="2">
+        <v>0</v>
+      </c>
+      <c r="R9" s="2">
         <v>14</v>
       </c>
-      <c r="Q9" s="14">
+      <c r="S9" s="11">
         <f t="shared" si="0"/>
         <v>59</v>
       </c>
-      <c r="S9" s="9"/>
+      <c r="U9" s="6"/>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="11">
-        <v>45635</v>
+      <c r="B10" s="8">
+        <v>45269</v>
       </c>
       <c r="C10" s="2">
         <v>15</v>
@@ -1206,20 +1260,26 @@
         <v>0</v>
       </c>
       <c r="P10" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="2">
+        <v>0</v>
+      </c>
+      <c r="R10" s="2">
         <v>1</v>
       </c>
-      <c r="Q10" s="14">
+      <c r="S10" s="11">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="S10" s="8"/>
+      <c r="U10" s="5"/>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="11">
-        <v>45629</v>
+      <c r="B11" s="8">
+        <v>45263</v>
       </c>
       <c r="C11" s="2">
         <v>25</v>
@@ -1261,20 +1321,26 @@
         <v>0</v>
       </c>
       <c r="P11" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="2">
+        <v>0</v>
+      </c>
+      <c r="R11" s="2">
         <v>1</v>
       </c>
-      <c r="Q11" s="14">
+      <c r="S11" s="11">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="S11" s="8"/>
+      <c r="U11" s="5"/>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="11">
-        <v>45636</v>
+      <c r="B12" s="8">
+        <v>45270</v>
       </c>
       <c r="C12" s="2">
         <v>25</v>
@@ -1316,22 +1382,28 @@
         <v>0</v>
       </c>
       <c r="P12" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="2">
+        <v>0</v>
+      </c>
+      <c r="R12" s="2">
         <v>3</v>
       </c>
-      <c r="Q12" s="14">
+      <c r="S12" s="11">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="S12" s="8"/>
+      <c r="U12" s="5"/>
     </row>
-    <row r="13" spans="1:19" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:21" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="11">
-        <v>45628</v>
-      </c>
-      <c r="C13" s="5">
+      <c r="B13" s="8">
+        <v>45262</v>
+      </c>
+      <c r="C13" s="2">
         <v>10</v>
       </c>
       <c r="D13" s="2">
@@ -1343,48 +1415,54 @@
       <c r="F13" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="2">
         <v>9</v>
       </c>
-      <c r="H13" s="5">
-        <v>0</v>
-      </c>
-      <c r="I13" s="5">
+      <c r="H13" s="2">
+        <v>0</v>
+      </c>
+      <c r="I13" s="2">
         <v>9</v>
       </c>
-      <c r="J13" s="5">
-        <v>0</v>
-      </c>
-      <c r="K13" s="5">
-        <v>0</v>
-      </c>
-      <c r="L13" s="5">
-        <v>0</v>
-      </c>
-      <c r="M13" s="5">
-        <v>0</v>
-      </c>
-      <c r="N13" s="5">
+      <c r="J13" s="2">
+        <v>0</v>
+      </c>
+      <c r="K13" s="2">
+        <v>0</v>
+      </c>
+      <c r="L13" s="2">
+        <v>0</v>
+      </c>
+      <c r="M13" s="2">
+        <v>0</v>
+      </c>
+      <c r="N13" s="2">
         <v>6</v>
       </c>
-      <c r="O13" s="5">
-        <v>0</v>
-      </c>
-      <c r="P13" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="14">
+      <c r="O13" s="2">
+        <v>0</v>
+      </c>
+      <c r="P13" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="2">
+        <v>0</v>
+      </c>
+      <c r="R13" s="2">
+        <v>0</v>
+      </c>
+      <c r="S13" s="11">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="S13" s="9"/>
+      <c r="U13" s="6"/>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="11">
-        <v>45636</v>
+      <c r="B14" s="8">
+        <v>45270</v>
       </c>
       <c r="C14" s="2">
         <v>40</v>
@@ -1426,22 +1504,28 @@
         <v>0</v>
       </c>
       <c r="P14" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="2">
+        <v>0</v>
+      </c>
+      <c r="R14" s="2">
         <v>5</v>
       </c>
-      <c r="Q14" s="14">
+      <c r="S14" s="11">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="S14" s="8"/>
+      <c r="U14" s="5"/>
     </row>
-    <row r="15" spans="1:19" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:21" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A15" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="11">
-        <v>45635</v>
-      </c>
-      <c r="C15" s="5">
+      <c r="B15" s="8">
+        <v>45269</v>
+      </c>
+      <c r="C15" s="2">
         <v>30</v>
       </c>
       <c r="D15" s="2">
@@ -1453,41 +1537,47 @@
       <c r="F15" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="2">
         <v>22</v>
       </c>
-      <c r="H15" s="5">
-        <v>0</v>
-      </c>
-      <c r="I15" s="5">
+      <c r="H15" s="2">
+        <v>0</v>
+      </c>
+      <c r="I15" s="2">
         <v>22</v>
       </c>
-      <c r="J15" s="5">
-        <v>0</v>
-      </c>
-      <c r="K15" s="5">
-        <v>0</v>
-      </c>
-      <c r="L15" s="5">
+      <c r="J15" s="2">
+        <v>0</v>
+      </c>
+      <c r="K15" s="2">
+        <v>0</v>
+      </c>
+      <c r="L15" s="2">
         <v>2</v>
       </c>
-      <c r="M15" s="5">
+      <c r="M15" s="2">
         <v>2</v>
       </c>
-      <c r="N15" s="5">
+      <c r="N15" s="2">
         <v>11</v>
       </c>
-      <c r="O15" s="5">
-        <v>0</v>
-      </c>
-      <c r="P15" s="6">
+      <c r="O15" s="2">
+        <v>0</v>
+      </c>
+      <c r="P15" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="2">
+        <v>0</v>
+      </c>
+      <c r="R15" s="2">
         <v>2</v>
       </c>
-      <c r="Q15" s="14">
+      <c r="S15" s="11">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="S15" s="9"/>
+      <c r="U15" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>